<commit_message>
Project5 implementation feedback Isabella
</commit_message>
<xml_diff>
--- a/data/data_raw.xlsx
+++ b/data/data_raw.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Bootcamp\6_Projects\Proj5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Bootcamp\6_Projects\Proj5_Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC1FC941-ED17-4A22-A504-9B5EC390478B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F78AFE-F50D-4525-80DE-4714590CC8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10716" yWindow="0" windowWidth="12384" windowHeight="12336" xr2:uid="{135B64BA-8E2C-4F42-A65B-386A4D268FDB}"/>
+    <workbookView xWindow="-19310" yWindow="750" windowWidth="19420" windowHeight="10300" xr2:uid="{135B64BA-8E2C-4F42-A65B-386A4D268FDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -713,7 +713,7 @@
         <v>1.72</v>
       </c>
       <c r="L6" s="2">
-        <f t="shared" ref="L6:L8" si="3">M6-K6</f>
+        <f t="shared" ref="L6:L7" si="3">M6-K6</f>
         <v>4.8953846153846152</v>
       </c>
       <c r="M6" s="2">
@@ -934,6 +934,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D1" r:id="rId1" xr:uid="{754D97A5-6B07-462A-9769-63C58B3D82CE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>